<commit_message>
improved filters and ui
</commit_message>
<xml_diff>
--- a/Topics.xlsx
+++ b/Topics.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\james\OneDrive\Admin\WebApps\MathsDatabase\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/be3e99465cf27169/Admin/WebApps/MathsDatabase/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16C6499D-8C65-44BA-8AFC-36C43F997663}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="7" documentId="13_ncr:1_{16C6499D-8C65-44BA-8AFC-36C43F997663}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A83D1DED-8087-4B92-9214-F8160C1118A5}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="41496" windowHeight="17496" xr2:uid="{5F3515D1-ED24-4918-92E0-EFD994F45BDC}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="304" uniqueCount="174">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="310" uniqueCount="177">
   <si>
     <t>Topic</t>
   </si>
@@ -558,6 +558,15 @@
   </si>
   <si>
     <t>Measurement error</t>
+  </si>
+  <si>
+    <t>Transformations</t>
+  </si>
+  <si>
+    <t>Line and rotational symmetry</t>
+  </si>
+  <si>
+    <t>Bivariate data</t>
   </si>
 </sst>
 </file>
@@ -929,7 +938,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9BC17005-3F68-4D76-AB6F-A3AD581A36F2}">
-  <dimension ref="A1:B152"/>
+  <dimension ref="A1:B155"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="22.77734375" customWidth="1"/>
@@ -2152,6 +2161,30 @@
         <v>168</v>
       </c>
     </row>
+    <row r="153" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A153" t="s">
+        <v>64</v>
+      </c>
+      <c r="B153" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="154" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A154" t="s">
+        <v>13</v>
+      </c>
+      <c r="B154" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="155" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A155" t="s">
+        <v>22</v>
+      </c>
+      <c r="B155" t="s">
+        <v>176</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
added subtopic, improved worksheet generation
</commit_message>
<xml_diff>
--- a/Topics.xlsx
+++ b/Topics.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29825"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/be3e99465cf27169/Admin/WebApps/MathsDatabase/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\james\OneDrive\Admin\WebApps\MathsDatabase\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="7" documentId="13_ncr:1_{16C6499D-8C65-44BA-8AFC-36C43F997663}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A83D1DED-8087-4B92-9214-F8160C1118A5}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4EED1BC-4977-40E2-A8B7-5E0BA3E57ACC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="41496" windowHeight="17496" xr2:uid="{5F3515D1-ED24-4918-92E0-EFD994F45BDC}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="310" uniqueCount="177">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="312" uniqueCount="178">
   <si>
     <t>Topic</t>
   </si>
@@ -567,13 +567,16 @@
   </si>
   <si>
     <t>Bivariate data</t>
+  </si>
+  <si>
+    <t>Inverse functions</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -938,14 +941,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9BC17005-3F68-4D76-AB6F-A3AD581A36F2}">
-  <dimension ref="A1:B155"/>
-  <sheetFormatPr defaultRowHeight="14.45"/>
+  <dimension ref="A1:B156"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="22.7109375" customWidth="1"/>
-    <col min="2" max="2" width="33.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="22.6640625" customWidth="1"/>
+    <col min="2" max="2" width="33.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -953,7 +956,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -961,7 +964,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:2">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>2</v>
       </c>
@@ -969,7 +972,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:2">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>2</v>
       </c>
@@ -977,7 +980,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:2">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>2</v>
       </c>
@@ -985,7 +988,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="1:2">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>2</v>
       </c>
@@ -993,7 +996,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="7" spans="1:2">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>2</v>
       </c>
@@ -1001,7 +1004,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="8" spans="1:2">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>2</v>
       </c>
@@ -1009,7 +1012,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="9" spans="1:2">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>2</v>
       </c>
@@ -1017,7 +1020,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="10" spans="1:2">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>2</v>
       </c>
@@ -1025,7 +1028,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="11" spans="1:2">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>12</v>
       </c>
@@ -1033,7 +1036,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="12" spans="1:2">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>12</v>
       </c>
@@ -1041,7 +1044,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="13" spans="1:2">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>12</v>
       </c>
@@ -1049,7 +1052,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="14" spans="1:2">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>16</v>
       </c>
@@ -1057,7 +1060,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="15" spans="1:2">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>16</v>
       </c>
@@ -1065,7 +1068,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="16" spans="1:2">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>16</v>
       </c>
@@ -1073,7 +1076,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="17" spans="1:2">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>16</v>
       </c>
@@ -1081,7 +1084,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="18" spans="1:2">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>21</v>
       </c>
@@ -1089,7 +1092,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="19" spans="1:2">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>21</v>
       </c>
@@ -1097,7 +1100,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="20" spans="1:2">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>21</v>
       </c>
@@ -1105,7 +1108,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="21" spans="1:2">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>25</v>
       </c>
@@ -1113,7 +1116,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="22" spans="1:2">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>25</v>
       </c>
@@ -1121,7 +1124,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="23" spans="1:2">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>2</v>
       </c>
@@ -1129,7 +1132,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="24" spans="1:2">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>2</v>
       </c>
@@ -1137,7 +1140,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="25" spans="1:2">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>2</v>
       </c>
@@ -1145,7 +1148,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="26" spans="1:2">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>12</v>
       </c>
@@ -1153,7 +1156,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="27" spans="1:2">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>12</v>
       </c>
@@ -1161,7 +1164,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="28" spans="1:2">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>12</v>
       </c>
@@ -1169,7 +1172,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="29" spans="1:2">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>34</v>
       </c>
@@ -1177,7 +1180,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="30" spans="1:2">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>34</v>
       </c>
@@ -1185,7 +1188,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="31" spans="1:2">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>34</v>
       </c>
@@ -1193,7 +1196,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="32" spans="1:2">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>34</v>
       </c>
@@ -1201,7 +1204,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="33" spans="1:2">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>34</v>
       </c>
@@ -1209,7 +1212,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="34" spans="1:2">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>34</v>
       </c>
@@ -1217,7 +1220,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="35" spans="1:2">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>41</v>
       </c>
@@ -1225,7 +1228,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="36" spans="1:2">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>41</v>
       </c>
@@ -1233,7 +1236,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="37" spans="1:2">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>41</v>
       </c>
@@ -1241,7 +1244,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="38" spans="1:2">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>41</v>
       </c>
@@ -1249,7 +1252,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="39" spans="1:2">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>41</v>
       </c>
@@ -1257,7 +1260,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="40" spans="1:2">
+    <row r="40" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>41</v>
       </c>
@@ -1265,7 +1268,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="41" spans="1:2">
+    <row r="41" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>41</v>
       </c>
@@ -1273,7 +1276,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="42" spans="1:2">
+    <row r="42" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>41</v>
       </c>
@@ -1281,7 +1284,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="43" spans="1:2">
+    <row r="43" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>41</v>
       </c>
@@ -1289,7 +1292,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="44" spans="1:2">
+    <row r="44" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>41</v>
       </c>
@@ -1297,7 +1300,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="45" spans="1:2">
+    <row r="45" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>41</v>
       </c>
@@ -1305,7 +1308,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="46" spans="1:2">
+    <row r="46" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>41</v>
       </c>
@@ -1313,7 +1316,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="47" spans="1:2">
+    <row r="47" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>41</v>
       </c>
@@ -1321,7 +1324,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="48" spans="1:2">
+    <row r="48" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>41</v>
       </c>
@@ -1329,7 +1332,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="49" spans="1:2">
+    <row r="49" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
         <v>41</v>
       </c>
@@ -1337,7 +1340,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="50" spans="1:2">
+    <row r="50" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
         <v>57</v>
       </c>
@@ -1345,7 +1348,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="51" spans="1:2">
+    <row r="51" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
         <v>57</v>
       </c>
@@ -1353,7 +1356,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="52" spans="1:2">
+    <row r="52" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
         <v>57</v>
       </c>
@@ -1361,7 +1364,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="53" spans="1:2">
+    <row r="53" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
         <v>57</v>
       </c>
@@ -1369,7 +1372,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="54" spans="1:2">
+    <row r="54" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
         <v>57</v>
       </c>
@@ -1377,7 +1380,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="55" spans="1:2">
+    <row r="55" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
         <v>57</v>
       </c>
@@ -1385,7 +1388,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="56" spans="1:2">
+    <row r="56" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
         <v>64</v>
       </c>
@@ -1393,7 +1396,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="57" spans="1:2">
+    <row r="57" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
         <v>66</v>
       </c>
@@ -1401,7 +1404,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="58" spans="1:2">
+    <row r="58" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
         <v>66</v>
       </c>
@@ -1409,7 +1412,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="59" spans="1:2">
+    <row r="59" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
         <v>66</v>
       </c>
@@ -1417,7 +1420,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="60" spans="1:2">
+    <row r="60" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
         <v>66</v>
       </c>
@@ -1425,7 +1428,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="61" spans="1:2">
+    <row r="61" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
         <v>66</v>
       </c>
@@ -1433,7 +1436,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="62" spans="1:2">
+    <row r="62" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
         <v>66</v>
       </c>
@@ -1441,7 +1444,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="63" spans="1:2">
+    <row r="63" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
         <v>12</v>
       </c>
@@ -1449,7 +1452,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="64" spans="1:2">
+    <row r="64" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
         <v>12</v>
       </c>
@@ -1457,7 +1460,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="65" spans="1:2">
+    <row r="65" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
         <v>12</v>
       </c>
@@ -1465,7 +1468,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="66" spans="1:2">
+    <row r="66" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
         <v>12</v>
       </c>
@@ -1473,7 +1476,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="67" spans="1:2">
+    <row r="67" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
         <v>12</v>
       </c>
@@ -1481,7 +1484,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="68" spans="1:2">
+    <row r="68" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
         <v>12</v>
       </c>
@@ -1489,7 +1492,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="69" spans="1:2">
+    <row r="69" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
         <v>16</v>
       </c>
@@ -1497,7 +1500,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="70" spans="1:2">
+    <row r="70" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
         <v>16</v>
       </c>
@@ -1505,7 +1508,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="71" spans="1:2">
+    <row r="71" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
         <v>16</v>
       </c>
@@ -1513,7 +1516,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="72" spans="1:2">
+    <row r="72" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
         <v>16</v>
       </c>
@@ -1521,7 +1524,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="73" spans="1:2">
+    <row r="73" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
         <v>16</v>
       </c>
@@ -1529,7 +1532,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="74" spans="1:2">
+    <row r="74" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
         <v>16</v>
       </c>
@@ -1537,7 +1540,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="75" spans="1:2">
+    <row r="75" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
         <v>21</v>
       </c>
@@ -1545,7 +1548,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="76" spans="1:2">
+    <row r="76" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
         <v>21</v>
       </c>
@@ -1553,7 +1556,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="77" spans="1:2">
+    <row r="77" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
         <v>21</v>
       </c>
@@ -1561,7 +1564,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="78" spans="1:2">
+    <row r="78" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
         <v>21</v>
       </c>
@@ -1569,7 +1572,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="79" spans="1:2">
+    <row r="79" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
         <v>21</v>
       </c>
@@ -1577,7 +1580,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="80" spans="1:2">
+    <row r="80" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
         <v>21</v>
       </c>
@@ -1585,7 +1588,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="81" spans="1:2">
+    <row r="81" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
         <v>21</v>
       </c>
@@ -1593,7 +1596,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="82" spans="1:2">
+    <row r="82" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
         <v>21</v>
       </c>
@@ -1601,7 +1604,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="83" spans="1:2">
+    <row r="83" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A83" t="s">
         <v>21</v>
       </c>
@@ -1609,7 +1612,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="84" spans="1:2">
+    <row r="84" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
         <v>94</v>
       </c>
@@ -1617,7 +1620,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="85" spans="1:2">
+    <row r="85" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
         <v>94</v>
       </c>
@@ -1625,7 +1628,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="86" spans="1:2">
+    <row r="86" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
         <v>94</v>
       </c>
@@ -1633,7 +1636,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="87" spans="1:2">
+    <row r="87" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A87" t="s">
         <v>94</v>
       </c>
@@ -1641,7 +1644,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="88" spans="1:2">
+    <row r="88" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A88" t="s">
         <v>25</v>
       </c>
@@ -1649,7 +1652,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="89" spans="1:2">
+    <row r="89" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A89" t="s">
         <v>25</v>
       </c>
@@ -1657,7 +1660,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="90" spans="1:2">
+    <row r="90" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A90" t="s">
         <v>25</v>
       </c>
@@ -1665,7 +1668,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="91" spans="1:2">
+    <row r="91" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A91" t="s">
         <v>25</v>
       </c>
@@ -1673,7 +1676,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="92" spans="1:2">
+    <row r="92" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A92" t="s">
         <v>103</v>
       </c>
@@ -1681,7 +1684,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="93" spans="1:2">
+    <row r="93" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A93" t="s">
         <v>103</v>
       </c>
@@ -1689,7 +1692,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="94" spans="1:2">
+    <row r="94" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A94" t="s">
         <v>103</v>
       </c>
@@ -1697,7 +1700,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="95" spans="1:2">
+    <row r="95" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A95" t="s">
         <v>103</v>
       </c>
@@ -1705,7 +1708,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="96" spans="1:2">
+    <row r="96" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A96" t="s">
         <v>103</v>
       </c>
@@ -1713,7 +1716,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="97" spans="1:2">
+    <row r="97" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A97" t="s">
         <v>103</v>
       </c>
@@ -1721,7 +1724,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="98" spans="1:2">
+    <row r="98" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A98" t="s">
         <v>103</v>
       </c>
@@ -1729,7 +1732,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="99" spans="1:2">
+    <row r="99" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A99" t="s">
         <v>103</v>
       </c>
@@ -1737,7 +1740,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="100" spans="1:2">
+    <row r="100" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A100" t="s">
         <v>103</v>
       </c>
@@ -1745,7 +1748,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="101" spans="1:2">
+    <row r="101" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A101" t="s">
         <v>113</v>
       </c>
@@ -1753,7 +1756,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="102" spans="1:2">
+    <row r="102" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A102" t="s">
         <v>113</v>
       </c>
@@ -1761,7 +1764,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="103" spans="1:2">
+    <row r="103" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A103" t="s">
         <v>113</v>
       </c>
@@ -1769,7 +1772,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="104" spans="1:2">
+    <row r="104" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A104" t="s">
         <v>34</v>
       </c>
@@ -1777,7 +1780,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="105" spans="1:2">
+    <row r="105" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A105" t="s">
         <v>34</v>
       </c>
@@ -1785,7 +1788,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="106" spans="1:2">
+    <row r="106" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A106" t="s">
         <v>34</v>
       </c>
@@ -1793,7 +1796,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="107" spans="1:2">
+    <row r="107" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A107" t="s">
         <v>34</v>
       </c>
@@ -1801,7 +1804,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="108" spans="1:2">
+    <row r="108" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A108" t="s">
         <v>34</v>
       </c>
@@ -1809,7 +1812,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="109" spans="1:2">
+    <row r="109" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A109" t="s">
         <v>41</v>
       </c>
@@ -1817,7 +1820,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="110" spans="1:2">
+    <row r="110" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A110" t="s">
         <v>41</v>
       </c>
@@ -1825,7 +1828,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="111" spans="1:2">
+    <row r="111" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A111" t="s">
         <v>41</v>
       </c>
@@ -1833,7 +1836,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="112" spans="1:2">
+    <row r="112" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A112" t="s">
         <v>41</v>
       </c>
@@ -1841,7 +1844,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="113" spans="1:2">
+    <row r="113" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A113" t="s">
         <v>41</v>
       </c>
@@ -1849,7 +1852,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="114" spans="1:2">
+    <row r="114" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A114" t="s">
         <v>41</v>
       </c>
@@ -1857,7 +1860,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="115" spans="1:2">
+    <row r="115" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A115" t="s">
         <v>128</v>
       </c>
@@ -1865,7 +1868,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="116" spans="1:2">
+    <row r="116" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A116" t="s">
         <v>128</v>
       </c>
@@ -1873,7 +1876,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="117" spans="1:2">
+    <row r="117" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A117" t="s">
         <v>131</v>
       </c>
@@ -1881,7 +1884,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="118" spans="1:2">
+    <row r="118" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A118" t="s">
         <v>131</v>
       </c>
@@ -1889,7 +1892,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="119" spans="1:2">
+    <row r="119" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A119" t="s">
         <v>131</v>
       </c>
@@ -1897,7 +1900,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="120" spans="1:2">
+    <row r="120" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A120" t="s">
         <v>131</v>
       </c>
@@ -1905,7 +1908,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="121" spans="1:2">
+    <row r="121" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A121" t="s">
         <v>131</v>
       </c>
@@ -1913,7 +1916,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="122" spans="1:2">
+    <row r="122" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A122" t="s">
         <v>131</v>
       </c>
@@ -1921,7 +1924,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="123" spans="1:2">
+    <row r="123" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A123" t="s">
         <v>131</v>
       </c>
@@ -1929,7 +1932,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="124" spans="1:2">
+    <row r="124" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A124" t="s">
         <v>131</v>
       </c>
@@ -1937,7 +1940,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="125" spans="1:2">
+    <row r="125" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A125" t="s">
         <v>131</v>
       </c>
@@ -1945,7 +1948,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="126" spans="1:2">
+    <row r="126" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A126" t="s">
         <v>131</v>
       </c>
@@ -1953,7 +1956,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="127" spans="1:2">
+    <row r="127" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A127" t="s">
         <v>131</v>
       </c>
@@ -1961,7 +1964,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="128" spans="1:2">
+    <row r="128" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A128" t="s">
         <v>64</v>
       </c>
@@ -1969,7 +1972,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="129" spans="1:2">
+    <row r="129" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A129" t="s">
         <v>64</v>
       </c>
@@ -1977,7 +1980,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="130" spans="1:2">
+    <row r="130" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A130" t="s">
         <v>64</v>
       </c>
@@ -1985,7 +1988,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="131" spans="1:2">
+    <row r="131" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A131" t="s">
         <v>64</v>
       </c>
@@ -1993,7 +1996,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="132" spans="1:2">
+    <row r="132" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A132" t="s">
         <v>64</v>
       </c>
@@ -2001,7 +2004,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="133" spans="1:2">
+    <row r="133" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A133" t="s">
         <v>148</v>
       </c>
@@ -2009,7 +2012,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="134" spans="1:2">
+    <row r="134" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A134" t="s">
         <v>148</v>
       </c>
@@ -2017,7 +2020,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="135" spans="1:2">
+    <row r="135" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A135" t="s">
         <v>151</v>
       </c>
@@ -2025,7 +2028,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="136" spans="1:2">
+    <row r="136" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A136" t="s">
         <v>151</v>
       </c>
@@ -2033,7 +2036,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="137" spans="1:2">
+    <row r="137" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A137" t="s">
         <v>154</v>
       </c>
@@ -2041,7 +2044,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="138" spans="1:2">
+    <row r="138" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A138" t="s">
         <v>154</v>
       </c>
@@ -2049,7 +2052,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="139" spans="1:2">
+    <row r="139" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A139" t="s">
         <v>154</v>
       </c>
@@ -2057,7 +2060,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="140" spans="1:2">
+    <row r="140" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A140" t="s">
         <v>154</v>
       </c>
@@ -2065,7 +2068,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="141" spans="1:2">
+    <row r="141" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A141" t="s">
         <v>154</v>
       </c>
@@ -2073,7 +2076,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="142" spans="1:2">
+    <row r="142" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A142" t="s">
         <v>154</v>
       </c>
@@ -2081,7 +2084,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="143" spans="1:2">
+    <row r="143" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A143" t="s">
         <v>2</v>
       </c>
@@ -2089,7 +2092,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="144" spans="1:2">
+    <row r="144" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A144" t="s">
         <v>162</v>
       </c>
@@ -2097,7 +2100,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="145" spans="1:2">
+    <row r="145" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A145" t="s">
         <v>162</v>
       </c>
@@ -2105,7 +2108,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="146" spans="1:2">
+    <row r="146" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A146" t="s">
         <v>165</v>
       </c>
@@ -2113,7 +2116,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="147" spans="1:2">
+    <row r="147" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A147" t="s">
         <v>165</v>
       </c>
@@ -2121,7 +2124,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="148" spans="1:2">
+    <row r="148" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A148" t="s">
         <v>148</v>
       </c>
@@ -2129,7 +2132,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="149" spans="1:2">
+    <row r="149" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A149" t="s">
         <v>148</v>
       </c>
@@ -2137,7 +2140,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="150" spans="1:2">
+    <row r="150" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A150" t="s">
         <v>170</v>
       </c>
@@ -2145,7 +2148,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="151" spans="1:2">
+    <row r="151" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A151" t="s">
         <v>170</v>
       </c>
@@ -2153,7 +2156,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="152" spans="1:2">
+    <row r="152" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A152" t="s">
         <v>170</v>
       </c>
@@ -2161,7 +2164,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="153" spans="1:2">
+    <row r="153" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A153" t="s">
         <v>94</v>
       </c>
@@ -2169,7 +2172,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="154" spans="1:2">
+    <row r="154" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A154" t="s">
         <v>34</v>
       </c>
@@ -2177,12 +2180,20 @@
         <v>175</v>
       </c>
     </row>
-    <row r="155" spans="1:2">
+    <row r="155" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A155" t="s">
         <v>57</v>
       </c>
       <c r="B155" t="s">
         <v>176</v>
+      </c>
+    </row>
+    <row r="156" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A156" t="s">
+        <v>148</v>
+      </c>
+      <c r="B156" t="s">
+        <v>177</v>
       </c>
     </row>
   </sheetData>

</xml_diff>